<commit_message>
Garantizar lectura completa de filas sin omitir celdas vacias
</commit_message>
<xml_diff>
--- a/FORMATO DE CONTROL DE INVENTARIO GEVISE.xlsx
+++ b/FORMATO DE CONTROL DE INVENTARIO GEVISE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\INVENTARIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B133B6A1-7E05-4A7E-B9DA-556BA757FCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF19B12-DA6D-4245-9B30-9D80ABC956F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -407,12 +407,6 @@
     <t xml:space="preserve">OTROS: </t>
   </si>
   <si>
-    <t>NOMBRE: GERARDO CARRION</t>
-  </si>
-  <si>
-    <t>CARGO: COORDINADOR</t>
-  </si>
-  <si>
     <t>RADIO</t>
   </si>
   <si>
@@ -429,6 +423,12 @@
   </si>
   <si>
     <t>SILLA</t>
+  </si>
+  <si>
+    <t>CARGO:</t>
+  </si>
+  <si>
+    <t>NOMBRE:</t>
   </si>
 </sst>
 </file>
@@ -3138,13 +3138,13 @@
     <row r="8" spans="1:12" ht="22.5" customHeight="1">
       <c r="A8" s="86"/>
       <c r="B8" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" s="45" t="s">
         <v>97</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" s="45" t="s">
-        <v>99</v>
       </c>
       <c r="E8" s="45"/>
       <c r="F8" s="45"/>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="21" spans="1:11" ht="18" customHeight="1">
       <c r="A21" s="40" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B21" s="43"/>
       <c r="C21" s="43"/>
@@ -3445,7 +3445,7 @@
     </row>
     <row r="28" spans="1:11" ht="18" customHeight="1">
       <c r="A28" s="40" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="B28" s="43"/>
       <c r="C28" s="43"/>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="29" spans="1:11" ht="18" customHeight="1">
       <c r="A29" s="40" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B29" s="43"/>
       <c r="C29" s="43"/>
@@ -3475,7 +3475,7 @@
     </row>
     <row r="30" spans="1:11" ht="18" customHeight="1">
       <c r="A30" s="40" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="B30" s="43"/>
       <c r="C30" s="43"/>
@@ -3565,7 +3565,7 @@
     </row>
     <row r="36" spans="1:11" ht="18" customHeight="1">
       <c r="A36" s="40" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="43"/>
       <c r="C36" s="43"/>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="38" spans="1:11" ht="18" customHeight="1">
       <c r="A38" s="40" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B38" s="43"/>
       <c r="C38" s="43"/>
@@ -3757,7 +3757,7 @@
     </row>
     <row r="48" spans="1:11" ht="32.25" customHeight="1">
       <c r="A48" s="83" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B48" s="83"/>
       <c r="C48" s="83"/>
@@ -3774,7 +3774,7 @@
     </row>
     <row r="49" spans="1:11">
       <c r="A49" s="83" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B49" s="83"/>
       <c r="C49" s="83"/>

</xml_diff>